<commit_message>
Team Schedule Capture as of 10/28/2026 3:40 PM
</commit_message>
<xml_diff>
--- a/data/2026/cjsl/fall/brooklyn-city-fc-b13-14.xlsx
+++ b/data/2026/cjsl/fall/brooklyn-city-fc-b13-14.xlsx
@@ -74,7 +74,7 @@
     <col min="2" max="2" bestFit="1" customWidth="1" width="28.6"/>
     <col min="3" max="3" bestFit="1" customWidth="1" width="13.200000000000001"/>
     <col min="4" max="4" bestFit="1" customWidth="1" width="49.50000000000001"/>
-    <col min="5" max="5" bestFit="1" customWidth="1" width="7.700000000000001"/>
+    <col min="5" max="5" bestFit="1" customWidth="1" width="8.8"/>
     <col min="6" max="6" bestFit="1" customWidth="1" width="49.50000000000001"/>
     <col min="7" max="7" bestFit="1" customWidth="1" width="36.300000000000004"/>
     <col min="8" max="8" bestFit="1" customWidth="1" width="15.400000000000002"/>
@@ -329,7 +329,7 @@
       </c>
       <c r="E6" s="0" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>13 - 0</t>
         </is>
       </c>
       <c r="F6" s="0" t="inlineStr">

</xml_diff>